<commit_message>
fix: PDF liquidador como hoja Excel horizontal con logo Zurich correcto.
El PDF se genera desde la plantilla FORMATO_LIQUIDACION; se corrige el anclaje del logo para no deformarlo y se exporta la liquidación en landscape.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/Liquidador_plantilla.xlsx
+++ b/public/templates/Liquidador_plantilla.xlsx
@@ -1810,19 +1810,14 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>426720</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>128000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>36000</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>742949</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>137160</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="1333500" cy="828675"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -1853,7 +1848,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2306,6 +2301,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
@@ -2826,7 +2824,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>